<commit_message>
default to Aptos (#120)
</commit_message>
<xml_diff>
--- a/src/ExcelsiorOpenXml.Tests/HtmlTests.Test.verified.xlsx
+++ b/src/ExcelsiorOpenXml.Tests/HtmlTests.Test.verified.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb620bdb38f9446ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="DeterministicId2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12,6 +12,7 @@
   <x:fonts count="1">
     <x:font>
       <x:sz val="11"/>
+      <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
   <x:fills count="2">
@@ -64,7 +65,10 @@
       <x:c r="A2" s="2" t="inlineStr">
         <x:is>
           <x:r>
-            <x:t xml:space="preserve">● the value</x:t>
+            <x:t xml:space="preserve">● </x:t>
+          </x:r>
+          <x:r>
+            <x:t xml:space="preserve">the value</x:t>
           </x:r>
         </x:is>
       </x:c>

</xml_diff>